<commit_message>
Detail WillWay's September line items from the Chatwork messages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/willway_202609.xlsx
+++ b/invoice_agent/willway_202609.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MTG 他</t>
+          <t>定例MTG 他</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -510,7 +510,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>追加検証レポート納品</t>
+          <t>①追加検証レポート（4KW・3センテンスの調査）</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -542,7 +542,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>追加検証レポート（実データ版）納品</t>
+          <t>②追加検証レポート 実データ版（検索結果）</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -574,7 +574,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GEO対策レポート納品</t>
+          <t>③GEO対策レポート（御社でとるべき対策）</t>
         </is>
       </c>
       <c r="D5" t="n">

</xml_diff>